<commit_message>
SRS blog: update fee calculations and editorial polish
- Break out three strategies: Endowus 100% Aggressive (0.69% all-in),
  Fund-Smart Amundi MSCI World (0.40%), and IBKR VWRA (0.19%)
- Update all projection tables with recalculated numbers (6.948% vs 7.485%)
- SRS now never overtakes non-SRS (was +$1,485 in final year, now -$74,584)
- Update SRS balance at retirement ($1,800,622), withdrawal figures, and
  effective tax rate (~3.2%)
- Abbreviate 44-row table to key years with spreadsheet link
- Add reader map, financial disclaimer, and clarify SRS withdrawal rules
- Fix trailing whitespace and double blank lines

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/blog/2026-02-27-srs-calculations/SRS.xlsx
+++ b/content/blog/2026-02-27-srs-calculations/SRS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tzeus\OneDrive\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41176D59-B9A8-4244-9143-301832A950FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{592DC0AE-D5D8-4A44-9989-7F2AC4506671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{67DCB7C8-7F33-4D7A-AEE3-92B0723FEAC7}"/>
   </bookViews>
@@ -144,9 +144,6 @@
     <t>If 0.4% Endowus Fees</t>
   </si>
   <si>
-    <t>If lower-risk portfolio (5%)</t>
-  </si>
-  <si>
     <t>Play with setting these values in the G column</t>
   </si>
   <si>
@@ -163,6 +160,9 @@
   </si>
   <si>
     <t>Tax Brackets</t>
+  </si>
+  <si>
+    <t>If Endowus Fund-Smart</t>
   </si>
 </sst>
 </file>
@@ -503,23 +503,23 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -545,6 +545,101 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="medium">
+          <color indexed="64"/>
+        </top>
+        <bottom style="medium">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="13" formatCode="0%"/>
     </dxf>
     <dxf>
@@ -555,24 +650,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="3" formatCode="#,##0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -684,6 +761,24 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="thin">
@@ -711,13 +806,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color rgb="FF000000"/>
@@ -729,6 +817,13 @@
           <color rgb="FF000000"/>
         </top>
         <bottom style="medium">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
           <color rgb="FF000000"/>
         </bottom>
       </border>
@@ -751,101 +846,6 @@
           <color indexed="64"/>
         </horizontal>
       </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="medium">
-          <color indexed="64"/>
-        </top>
-        <bottom style="medium">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -982,133 +982,133 @@
                   <c:v>166304</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>348676.77760000003</c:v>
+                  <c:v>348335.85440000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>548419.62179743999</c:v>
+                  <c:v>547338.39310183993</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>766935.20271366311</c:v>
+                  <c:v>764648.78382551263</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1005723.5297223438</c:v>
+                  <c:v>1001693.7552148523</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1266381.7592763919</c:v>
+                  <c:v>1259988.622911084</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1550661.8284855143</c:v>
+                  <c:v>1541194.0832567466</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1860451.8012552338</c:v>
+                  <c:v>1847096.5385476977</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2197786.3644941282</c:v>
+                  <c:v>2179617.5341803599</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2564858.1320405407</c:v>
+                  <c:v>2540823.9027305744</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2964029.8184336089</c:v>
+                  <c:v>2932938.6678891089</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3397847.3494310873</c:v>
+                  <c:v>3358352.7651405428</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3869053.9813214699</c:v>
+                  <c:v>3819637.640330445</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4380588.3999881521</c:v>
+                  <c:v>4319541.6852122406</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4935625.2288003629</c:v>
+                  <c:v>4861028.9612034997</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5537593.1113652959</c:v>
+                  <c:v>5447295.2814197671</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>6190186.0201488752</c:v>
+                  <c:v>6081777.3317536255</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>6897383.6935883043</c:v>
+                  <c:v>6768170.7335253656</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>7663473.6454850258</c:v>
+                  <c:v>7510449.4587895209</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>8493074.8675997984</c:v>
+                  <c:v>8312886.6995568927</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>9391153.9082747586</c:v>
+                  <c:v>9180067.8523752633</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>10363050.258844756</c:v>
+                  <c:v>10116912.546149222</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>11414535.571074057</c:v>
+                  <c:v>11128730.197552633</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>12551827.238760276</c:v>
+                  <c:v>12221229.535110071</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>13781622.713336976</c:v>
+                  <c:v>13400548.525729097</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>15111136.459106945</c:v>
+                  <c:v>14673286.541994277</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>16548139.751108911</c:v>
+                  <c:v>16046538.937959194</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>18100881.988325201</c:v>
+                  <c:v>17527812.667821456</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>19778355.589390539</c:v>
+                  <c:v>19125285.222171023</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>21590258.905901067</c:v>
+                  <c:v>20847760.592736922</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>23547038.222884983</c:v>
+                  <c:v>22704703.880223405</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>25659945.317487363</c:v>
+                  <c:v>24706290.820920654</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>27941099.444769915</c:v>
+                  <c:v>26863461.021234341</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>30323269.7238805</c:v>
+                  <c:v>29091108.46845638</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>32888628.89745469</c:v>
+                  <c:v>31485495.327102989</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>35651264.191476732</c:v>
+                  <c:v>34059102.042119302</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>38626346.139609069</c:v>
+                  <c:v>36825343.219754584</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>41830211.889552779</c:v>
+                  <c:v>39798637.549535871</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>45280454.915667161</c:v>
+                  <c:v>42994482.959901288</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>48996021.630489737</c:v>
+                  <c:v>46429537.399232559</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>52997315.425682172</c:v>
+                  <c:v>50121705.663347773</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>57306308.713724904</c:v>
+                  <c:v>54090232.722032011</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>61946663.585618123</c:v>
+                  <c:v>58355804.031058766</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>66943861.747159928</c:v>
+                  <c:v>62940653.352566175</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1162,133 +1162,133 @@
                   <c:v>178850</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>374693.565</c:v>
+                  <c:v>374326.92249999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>588902.30014850001</c:v>
+                  <c:v>587740.09264912503</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>822954.58302991965</c:v>
+                  <c:v>820498.13458391209</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1078443.8003849206</c:v>
+                  <c:v>1074116.429877518</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1357087.2187529206</c:v>
+                  <c:v>1350225.1347722504</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1660735.5377957881</c:v>
+                  <c:v>1650577.7980307213</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1991383.1788114677</c:v>
+                  <c:v>1977060.6243725044</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2351179.3649844369</c:v>
+                  <c:v>2331702.4318291536</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2742440.0542685543</c:v>
+                  <c:v>2716685.3549683802</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3167641.7960609621</c:v>
+                  <c:v>3134337.35540692</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3629466.7138295891</c:v>
+                  <c:v>3587175.7701106672</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4130809.6330476543</c:v>
+                  <c:v>4077912.8054280207</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4674789.5613320805</c:v>
+                  <c:v>4609465.2464173697</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>5264766.959451641</c:v>
+                  <c:v>5184969.8009648332</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5904362.3411036571</c:v>
+                  <c:v>5807799.5930372365</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>6597476.3036541166</c:v>
+                  <c:v>6481581.8910956625</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>7348310.8584759058</c:v>
+                  <c:v>7210216.9227149617</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>8161365.3631049069</c:v>
+                  <c:v>7997871.0589923812</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9041514.147132121</c:v>
+                  <c:v>8849051.4953624085</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>9994008.168403117</c:v>
+                  <c:v>9768604.5831468217</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>11024504.011576986</c:v>
+                  <c:v>10761741.25121903</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>12139095.117391396</c:v>
+                  <c:v>11834064.331196917</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>13344345.414189417</c:v>
+                  <c:v>12991597.92865763</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>14647291.787458716</c:v>
+                  <c:v>14240785.244535789</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>16055453.061050788</c:v>
+                  <c:v>15588492.555225791</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>17577020.627284825</c:v>
+                  <c:v>17042194.448823672</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>19220817.803879041</c:v>
+                  <c:v>18609926.99367414</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>20996348.469160471</c:v>
+                  <c:v>20300329.805313781</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>22913849.438125309</c:v>
+                  <c:v>22122691.262927916</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>24984346.867037266</c:v>
+                  <c:v>24086997.111078195</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>27219716.996374957</c:v>
+                  <c:v>26203982.700104926</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>29632751.565763965</c:v>
+                  <c:v>28485189.137575556</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>31911510.161171213</c:v>
+                  <c:v>30617305.54452309</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>34365505.292565279</c:v>
+                  <c:v>32909010.864530645</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>37008212.649563551</c:v>
+                  <c:v>35372250.327740766</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>39854144.202314988</c:v>
+                  <c:v>38019863.264772162</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>42918927.89147301</c:v>
+                  <c:v>40865650.030140363</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>46219393.446327284</c:v>
+                  <c:v>43924443.934896372</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>49773664.802349851</c:v>
+                  <c:v>47212188.563423373</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>53601259.625650555</c:v>
+                  <c:v>50746020.877395615</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>57723196.490863077</c:v>
+                  <c:v>54544360.540068679</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>62162110.301010445</c:v>
+                  <c:v>58627005.926492825</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>66942376.583158143</c:v>
+                  <c:v>63015237.320090815</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1296,7 +1296,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000063-4862-4D12-B45C-046DA3D755A1}"/>
+              <c16:uniqueId val="{00000030-4862-4D12-B45C-046DA3D755A1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1758,133 +1758,133 @@
                   <c:v>-12546</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-26016.787399999972</c:v>
+                  <c:v>-25991.068099999975</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-40482.678351060022</c:v>
+                  <c:v>-40401.699547285098</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-56019.380316256545</c:v>
+                  <c:v>-55849.350758399465</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-72720.270662576775</c:v>
+                  <c:v>-72422.674662665697</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-90705.459476528689</c:v>
+                  <c:v>-90236.511861166451</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-110073.70931027387</c:v>
+                  <c:v>-109383.71477397461</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-130931.3775562339</c:v>
+                  <c:v>-129964.08582480671</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-153393.00049030874</c:v>
+                  <c:v>-152084.89764879365</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-177581.92222801363</c:v>
+                  <c:v>-175861.45223780582</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-203611.97762735328</c:v>
+                  <c:v>-201398.68751781108</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-231619.36439850181</c:v>
+                  <c:v>-228823.00497012446</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-261755.65172618441</c:v>
+                  <c:v>-258275.16509757563</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-294201.16134392843</c:v>
+                  <c:v>-289923.56120512914</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-329141.73065127805</c:v>
+                  <c:v>-323940.83976133354</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-366769.2297383612</c:v>
+                  <c:v>-360504.31161746942</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-407290.28350524139</c:v>
+                  <c:v>-399804.55934203696</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-450927.16488760151</c:v>
+                  <c:v>-442046.1891895961</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-497891.71761988103</c:v>
+                  <c:v>-487421.60020286031</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-548439.27953232266</c:v>
+                  <c:v>-536164.79580551572</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-602854.26012835838</c:v>
+                  <c:v>-588536.73077155836</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-661453.75273223035</c:v>
+                  <c:v>-644828.70506980829</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-724559.54631733894</c:v>
+                  <c:v>-705334.13364428468</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-792518.17542914115</c:v>
+                  <c:v>-770368.39354755916</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-865669.07412173972</c:v>
+                  <c:v>-840236.71880669147</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-944316.60194384307</c:v>
+                  <c:v>-915206.01323151402</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-1028880.876175914</c:v>
+                  <c:v>-995655.5108644776</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>-1119935.8155538402</c:v>
+                  <c:v>-1082114.3258526847</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>-1217992.8797699325</c:v>
+                  <c:v>-1175044.5831427574</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>-1323590.5322242416</c:v>
+                  <c:v>-1274930.6701909937</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>-1437308.6441522837</c:v>
+                  <c:v>-1382293.2308547907</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>-1559771.6788875945</c:v>
+                  <c:v>-1497691.8791842721</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>-1691652.1209940501</c:v>
+                  <c:v>-1621728.1163412146</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>-1588240.4372907132</c:v>
+                  <c:v>-1526197.0760667101</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>-1476876.3951105885</c:v>
+                  <c:v>-1423515.5374276564</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>-1356948.4580868185</c:v>
+                  <c:v>-1313148.2856214643</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>-1227798.0627059191</c:v>
+                  <c:v>-1194520.0450175777</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>-1088716.0019202307</c:v>
+                  <c:v>-1067012.4806044921</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>-938938.53066012263</c:v>
+                  <c:v>-929960.97499508411</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>-777643.17186011374</c:v>
+                  <c:v>-782651.1641908139</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>-603944.19996838272</c:v>
+                  <c:v>-624315.21404784173</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>-416887.77713817358</c:v>
+                  <c:v>-454127.818036668</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>-215446.71539232135</c:v>
+                  <c:v>-271201.8954340592</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>1485.1640017852187</c:v>
+                  <c:v>-74583.967524640262</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3417,15 +3417,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>307044</xdr:colOff>
+      <xdr:colOff>385485</xdr:colOff>
       <xdr:row>49</xdr:row>
-      <xdr:rowOff>158562</xdr:rowOff>
+      <xdr:rowOff>180973</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>241490</xdr:colOff>
+      <xdr:colOff>319931</xdr:colOff>
       <xdr:row>86</xdr:row>
-      <xdr:rowOff>53787</xdr:rowOff>
+      <xdr:rowOff>76198</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3492,10 +3492,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6E97861E-0382-41D3-B2A0-4526B1B33216}" name="Table36" displayName="Table36" ref="F5:G14" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6E97861E-0382-41D3-B2A0-4526B1B33216}" name="Table36" displayName="Table36" ref="F5:G14" totalsRowShown="0" headerRowDxfId="22" headerRowBorderDxfId="21" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="F5:G14" xr:uid="{EA087177-F272-428E-904C-CCBBD5D5E8B6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{631F5A8D-1C7E-4062-B0AB-DE44ED12EC6B}" name="Constants" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{631F5A8D-1C7E-4062-B0AB-DE44ED12EC6B}" name="Constants" dataDxfId="18"/>
     <tableColumn id="2" xr3:uid="{67B516E5-59F6-435B-8852-ACC8833D8906}" name="Value" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3503,12 +3503,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2E15315B-9726-4F22-AF07-6536B6C547CA}" name="Table6" displayName="Table6" ref="I5:K14" totalsRowShown="0" dataDxfId="5" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2E15315B-9726-4F22-AF07-6536B6C547CA}" name="Table6" displayName="Table6" ref="I5:K14" totalsRowShown="0" dataDxfId="17" tableBorderDxfId="16">
   <autoFilter ref="I5:K14" xr:uid="{2E15315B-9726-4F22-AF07-6536B6C547CA}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{01404DB3-E83D-4E7F-B287-DFC6CDAE3123}" name="If Zero Endowus Fees" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{5EB4CA42-4CDF-44D4-986C-07D04C1EF989}" name="If 0.4% Endowus Fees" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{B82EECD2-74D7-4326-B5B0-CED039473315}" name="If lower-risk portfolio (5%)" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{01404DB3-E83D-4E7F-B287-DFC6CDAE3123}" name="If Zero Endowus Fees" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{5EB4CA42-4CDF-44D4-986C-07D04C1EF989}" name="If 0.4% Endowus Fees" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{B82EECD2-74D7-4326-B5B0-CED039473315}" name="If Endowus Fund-Smart" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3518,10 +3518,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{2A48A046-10A7-418E-9254-252E686B45DB}" name="Table8" displayName="Table8" ref="F17:I30" totalsRowShown="0">
   <autoFilter ref="F17:I30" xr:uid="{2A48A046-10A7-418E-9254-252E686B45DB}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{9FA0EE7F-C168-45F6-B1E4-F8321C025CEB}" name="Lower Bound ($)" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{E792E839-9304-43A6-BDBD-A4D5E4CCD20B}" name="Upper Bound ($)" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{76BC44D5-41D9-4145-92E1-60480654C28B}" name="Base Tax at Lower Bound ($)" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{C86A200E-A1B9-45DB-A077-292BA3F74643}" name="Tax Rate on Excess (%)" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{9FA0EE7F-C168-45F6-B1E4-F8321C025CEB}" name="Lower Bound ($)" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{E792E839-9304-43A6-BDBD-A4D5E4CCD20B}" name="Upper Bound ($)" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{76BC44D5-41D9-4145-92E1-60480654C28B}" name="Base Tax at Lower Bound ($)" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{C86A200E-A1B9-45DB-A077-292BA3F74643}" name="Tax Rate on Excess (%)" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3545,7 +3545,7 @@
     <tableColumn id="6" xr3:uid="{247509A9-74B0-4B31-8A8D-B6065BE02714}" name="SRS accumulated value">
       <calculatedColumnFormula>(G3+E4)*Result!$G$12</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D0F5E3B0-C659-41D7-B525-DDD87BE0D38B}" name="Personal account accumulated value" dataDxfId="22">
+    <tableColumn id="7" xr3:uid="{D0F5E3B0-C659-41D7-B525-DDD87BE0D38B}" name="Personal account accumulated value" dataDxfId="8">
       <calculatedColumnFormula>H3*Result!$G$13+D4+(-1*E4)+F4</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3554,11 +3554,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EA087177-F272-428E-904C-CCBBD5D5E8B6}" name="Table3" displayName="Table3" ref="J5:K14" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18" totalsRowBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EA087177-F272-428E-904C-CCBBD5D5E8B6}" name="Table3" displayName="Table3" ref="J5:K14" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="J5:K14" xr:uid="{EA087177-F272-428E-904C-CCBBD5D5E8B6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DB6D026F-D8BF-4630-BACA-C25136C7D650}" name="Constants" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{18242A12-065E-4DAF-A793-13B0C99C977A}" name="Value" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{DB6D026F-D8BF-4630-BACA-C25136C7D650}" name="Constants" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{18242A12-065E-4DAF-A793-13B0C99C977A}" name="Value" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3582,7 +3582,7 @@
     <tableColumn id="6" xr3:uid="{F36D6D7A-90BF-423D-AB99-B519D979DC0C}" name="SRS accumulated value">
       <calculatedColumnFormula>(G3+E4)*$K$12</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{9B8873A6-4156-43EB-9FC5-CAAAEDBCBDA0}" name="Personal account accumulated value" dataDxfId="21">
+    <tableColumn id="7" xr3:uid="{9B8873A6-4156-43EB-9FC5-CAAAEDBCBDA0}" name="Personal account accumulated value" dataDxfId="1">
       <calculatedColumnFormula>H3*$K$13+D4+(-1*E4)+F4</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3934,25 +3934,25 @@
         <f>B4-C4</f>
         <v>-12546</v>
       </c>
-      <c r="I4" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
+      <c r="I4" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
         <v>2025</v>
       </c>
       <c r="B5" s="17">
-        <v>348676.77760000003</v>
+        <v>348335.85440000001</v>
       </c>
       <c r="C5" s="17">
-        <v>374693.565</v>
+        <v>374326.92249999999</v>
       </c>
       <c r="D5" s="18">
-        <f t="shared" ref="D5:D47" si="0">B5-C5</f>
-        <v>-26016.787399999972</v>
+        <f t="shared" ref="D5:D10" si="0">B5-C5</f>
+        <v>-25991.068099999975</v>
       </c>
       <c r="F5" s="16" t="s">
         <v>4</v>
@@ -3967,7 +3967,7 @@
         <v>27</v>
       </c>
       <c r="K5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -3975,26 +3975,26 @@
         <v>2026</v>
       </c>
       <c r="B6" s="17">
-        <v>548419.62179743999</v>
+        <v>547338.39310183993</v>
       </c>
       <c r="C6" s="17">
-        <v>588902.30014850001</v>
+        <v>587740.09264912503</v>
       </c>
       <c r="D6" s="18">
         <f t="shared" si="0"/>
-        <v>-40482.678351060022</v>
+        <v>-40401.699547285098</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="21">
-        <v>0.12594169672084929</v>
+        <v>0.12437044863857565</v>
       </c>
       <c r="I6" s="21">
         <v>0.12812000000000001</v>
       </c>
       <c r="J6" s="21">
-        <v>0.12594169672084929</v>
+        <v>0.12437044863857565</v>
       </c>
       <c r="K6" s="21">
         <v>0.11258</v>
@@ -4005,14 +4005,14 @@
         <v>2027</v>
       </c>
       <c r="B7" s="17">
-        <v>766935.20271366311</v>
+        <v>764648.78382551263</v>
       </c>
       <c r="C7" s="17">
-        <v>822954.58302991965</v>
+        <v>820498.13458391209</v>
       </c>
       <c r="D7" s="18">
         <f t="shared" si="0"/>
-        <v>-56019.380316256545</v>
+        <v>-55849.350758399465</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>17</v>
@@ -4035,14 +4035,14 @@
         <v>2028</v>
       </c>
       <c r="B8" s="17">
-        <v>1005723.5297223438</v>
+        <v>1001693.7552148523</v>
       </c>
       <c r="C8" s="17">
-        <v>1078443.8003849206</v>
+        <v>1074116.429877518</v>
       </c>
       <c r="D8" s="18">
         <f t="shared" si="0"/>
-        <v>-72720.270662576775</v>
+        <v>-72422.674662665697</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>9</v>
@@ -4065,14 +4065,14 @@
         <v>2029</v>
       </c>
       <c r="B9" s="17">
-        <v>1266381.7592763919</v>
+        <v>1259988.622911084</v>
       </c>
       <c r="C9" s="17">
-        <v>1357087.2187529206</v>
+        <v>1350225.1347722504</v>
       </c>
       <c r="D9" s="18">
         <f t="shared" si="0"/>
-        <v>-90705.459476528689</v>
+        <v>-90236.511861166451</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>3</v>
@@ -4095,14 +4095,14 @@
         <v>2030</v>
       </c>
       <c r="B10" s="17">
-        <v>1550661.8284855143</v>
+        <v>1541194.0832567466</v>
       </c>
       <c r="C10" s="17">
-        <v>1660735.5377957881</v>
+        <v>1650577.7980307213</v>
       </c>
       <c r="D10" s="18">
         <f t="shared" si="0"/>
-        <v>-110073.70931027387</v>
+        <v>-109383.71477397461</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>8</v>
@@ -4125,14 +4125,14 @@
         <v>2031</v>
       </c>
       <c r="B11" s="17">
-        <v>1860451.8012552338</v>
+        <v>1847096.5385476977</v>
       </c>
       <c r="C11" s="17">
-        <v>1991383.1788114677</v>
+        <v>1977060.6243725044</v>
       </c>
       <c r="D11" s="18">
-        <f t="shared" si="0"/>
-        <v>-130931.3775562339</v>
+        <f>B11-C11</f>
+        <v>-129964.08582480671</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="24"/>
@@ -4145,33 +4145,30 @@
         <v>2032</v>
       </c>
       <c r="B12" s="17">
-        <v>2197786.3644941282</v>
+        <v>2179617.5341803599</v>
       </c>
       <c r="C12" s="17">
-        <v>2351179.3649844369</v>
+        <v>2331702.4318291536</v>
       </c>
       <c r="D12" s="18">
-        <f t="shared" si="0"/>
-        <v>-153393.00049030874</v>
+        <f>B12-C12</f>
+        <v>-152084.89764879365</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>6</v>
       </c>
       <c r="G12" s="22">
-        <f>MAX(G13*0.996, 1.04)</f>
-        <v>1.0725924</v>
+        <v>1.06948</v>
       </c>
       <c r="I12" s="22">
         <f>MAX(I13*1, 1.04)</f>
-        <v>1.0769</v>
+        <v>1.0748500000000001</v>
       </c>
       <c r="J12" s="22">
-        <f>MAX(J13*0.996, 1.04)</f>
-        <v>1.0725924</v>
+        <v>1.06948</v>
       </c>
       <c r="K12" s="22">
-        <f>MAX(K13*0.996, 1.04)</f>
-        <v>1.0458000000000001</v>
+        <v>1.0726</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -4179,29 +4176,29 @@
         <v>2033</v>
       </c>
       <c r="B13" s="17">
-        <v>2564858.1320405407</v>
+        <v>2540823.9027305744</v>
       </c>
       <c r="C13" s="17">
-        <v>2742440.0542685543</v>
+        <v>2716685.3549683802</v>
       </c>
       <c r="D13" s="18">
-        <f t="shared" si="0"/>
-        <v>-177581.92222801363</v>
+        <f>B13-C13</f>
+        <v>-175861.45223780582</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>7</v>
       </c>
       <c r="G13" s="22">
-        <v>1.0769</v>
+        <v>1.0748500000000001</v>
       </c>
       <c r="I13" s="22">
-        <v>1.0769</v>
+        <v>1.0748500000000001</v>
       </c>
       <c r="J13" s="22">
-        <v>1.0769</v>
+        <v>1.0748500000000001</v>
       </c>
       <c r="K13" s="22">
-        <v>1.05</v>
+        <v>1.0748500000000001</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -4209,14 +4206,14 @@
         <v>2034</v>
       </c>
       <c r="B14" s="17">
-        <v>2964029.8184336089</v>
+        <v>2932938.6678891089</v>
       </c>
       <c r="C14" s="17">
-        <v>3167641.7960609621</v>
+        <v>3134337.35540692</v>
       </c>
       <c r="D14" s="18">
-        <f t="shared" si="0"/>
-        <v>-203611.97762735328</v>
+        <f>B14-C14</f>
+        <v>-201398.68751781108</v>
       </c>
       <c r="F14" s="15" t="s">
         <v>13</v>
@@ -4239,14 +4236,14 @@
         <v>2035</v>
       </c>
       <c r="B15" s="17">
-        <v>3397847.3494310873</v>
+        <v>3358352.7651405428</v>
       </c>
       <c r="C15" s="17">
-        <v>3629466.7138295891</v>
+        <v>3587175.7701106672</v>
       </c>
       <c r="D15" s="18">
-        <f t="shared" si="0"/>
-        <v>-231619.36439850181</v>
+        <f>B15-C15</f>
+        <v>-228823.00497012446</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -4254,47 +4251,47 @@
         <v>2036</v>
       </c>
       <c r="B16" s="17">
-        <v>3869053.9813214699</v>
+        <v>3819637.640330445</v>
       </c>
       <c r="C16" s="17">
-        <v>4130809.6330476543</v>
+        <v>4077912.8054280207</v>
       </c>
       <c r="D16" s="18">
-        <f t="shared" si="0"/>
-        <v>-261755.65172618441</v>
-      </c>
-      <c r="F16" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
+        <f>B16-C16</f>
+        <v>-258275.16509757563</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
         <v>2037</v>
       </c>
       <c r="B17" s="17">
-        <v>4380588.3999881521</v>
+        <v>4319541.6852122406</v>
       </c>
       <c r="C17" s="17">
-        <v>4674789.5613320805</v>
+        <v>4609465.2464173697</v>
       </c>
       <c r="D17" s="18">
-        <f t="shared" si="0"/>
-        <v>-294201.16134392843</v>
+        <f>B17-C17</f>
+        <v>-289923.56120512914</v>
       </c>
       <c r="F17" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" t="s">
         <v>30</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>31</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>32</v>
-      </c>
-      <c r="I17" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -4302,25 +4299,25 @@
         <v>2038</v>
       </c>
       <c r="B18" s="17">
-        <v>4935625.2288003629</v>
+        <v>4861028.9612034997</v>
       </c>
       <c r="C18" s="17">
-        <v>5264766.959451641</v>
+        <v>5184969.8009648332</v>
       </c>
       <c r="D18" s="18">
-        <f t="shared" si="0"/>
-        <v>-329141.73065127805</v>
+        <f>B18-C18</f>
+        <v>-323940.83976133354</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
-      <c r="G18" s="28">
+      <c r="G18" s="26">
         <v>20000</v>
       </c>
-      <c r="H18" s="29">
-        <v>0</v>
-      </c>
-      <c r="I18" s="30">
+      <c r="H18" s="27">
+        <v>0</v>
+      </c>
+      <c r="I18" s="28">
         <v>0</v>
       </c>
     </row>
@@ -4329,25 +4326,25 @@
         <v>2039</v>
       </c>
       <c r="B19" s="17">
-        <v>5537593.1113652959</v>
+        <v>5447295.2814197671</v>
       </c>
       <c r="C19" s="17">
-        <v>5904362.3411036571</v>
+        <v>5807799.5930372365</v>
       </c>
       <c r="D19" s="18">
-        <f t="shared" si="0"/>
-        <v>-366769.2297383612</v>
-      </c>
-      <c r="F19" s="28">
+        <f>B19-C19</f>
+        <v>-360504.31161746942</v>
+      </c>
+      <c r="F19" s="26">
         <v>20000</v>
       </c>
-      <c r="G19" s="28">
+      <c r="G19" s="26">
         <v>30000</v>
       </c>
-      <c r="H19" s="29">
-        <v>0</v>
-      </c>
-      <c r="I19" s="30">
+      <c r="H19" s="27">
+        <v>0</v>
+      </c>
+      <c r="I19" s="28">
         <v>0.02</v>
       </c>
     </row>
@@ -4356,25 +4353,25 @@
         <v>2040</v>
       </c>
       <c r="B20" s="17">
-        <v>6190186.0201488752</v>
+        <v>6081777.3317536255</v>
       </c>
       <c r="C20" s="17">
-        <v>6597476.3036541166</v>
+        <v>6481581.8910956625</v>
       </c>
       <c r="D20" s="18">
-        <f t="shared" si="0"/>
-        <v>-407290.28350524139</v>
-      </c>
-      <c r="F20" s="28">
+        <f>B20-C20</f>
+        <v>-399804.55934203696</v>
+      </c>
+      <c r="F20" s="26">
         <v>30000</v>
       </c>
-      <c r="G20" s="28">
+      <c r="G20" s="26">
         <v>40000</v>
       </c>
-      <c r="H20" s="29">
+      <c r="H20" s="27">
         <v>200</v>
       </c>
-      <c r="I20" s="30">
+      <c r="I20" s="28">
         <v>0.04</v>
       </c>
     </row>
@@ -4383,25 +4380,25 @@
         <v>2041</v>
       </c>
       <c r="B21" s="17">
-        <v>6897383.6935883043</v>
+        <v>6768170.7335253656</v>
       </c>
       <c r="C21" s="17">
-        <v>7348310.8584759058</v>
+        <v>7210216.9227149617</v>
       </c>
       <c r="D21" s="18">
-        <f t="shared" si="0"/>
-        <v>-450927.16488760151</v>
-      </c>
-      <c r="F21" s="28">
+        <f>B21-C21</f>
+        <v>-442046.1891895961</v>
+      </c>
+      <c r="F21" s="26">
         <v>40000</v>
       </c>
-      <c r="G21" s="28">
+      <c r="G21" s="26">
         <v>80000</v>
       </c>
-      <c r="H21" s="29">
+      <c r="H21" s="27">
         <v>550</v>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="28">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
@@ -4410,25 +4407,25 @@
         <v>2042</v>
       </c>
       <c r="B22" s="17">
-        <v>7663473.6454850258</v>
+        <v>7510449.4587895209</v>
       </c>
       <c r="C22" s="17">
-        <v>8161365.3631049069</v>
+        <v>7997871.0589923812</v>
       </c>
       <c r="D22" s="18">
-        <f t="shared" si="0"/>
-        <v>-497891.71761988103</v>
-      </c>
-      <c r="F22" s="28">
+        <f>B22-C22</f>
+        <v>-487421.60020286031</v>
+      </c>
+      <c r="F22" s="26">
         <v>80000</v>
       </c>
-      <c r="G22" s="28">
+      <c r="G22" s="26">
         <v>120000</v>
       </c>
-      <c r="H22" s="29">
+      <c r="H22" s="27">
         <v>3350</v>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="28">
         <v>0.12</v>
       </c>
     </row>
@@ -4437,25 +4434,25 @@
         <v>2043</v>
       </c>
       <c r="B23" s="17">
-        <v>8493074.8675997984</v>
+        <v>8312886.6995568927</v>
       </c>
       <c r="C23" s="17">
-        <v>9041514.147132121</v>
+        <v>8849051.4953624085</v>
       </c>
       <c r="D23" s="18">
-        <f t="shared" si="0"/>
-        <v>-548439.27953232266</v>
-      </c>
-      <c r="F23" s="28">
+        <f>B23-C23</f>
+        <v>-536164.79580551572</v>
+      </c>
+      <c r="F23" s="26">
         <v>120000</v>
       </c>
-      <c r="G23" s="28">
+      <c r="G23" s="26">
         <v>160000</v>
       </c>
-      <c r="H23" s="29">
+      <c r="H23" s="27">
         <v>7950</v>
       </c>
-      <c r="I23" s="30">
+      <c r="I23" s="28">
         <v>0.15</v>
       </c>
     </row>
@@ -4464,25 +4461,25 @@
         <v>2044</v>
       </c>
       <c r="B24" s="17">
-        <v>9391153.9082747586</v>
+        <v>9180067.8523752633</v>
       </c>
       <c r="C24" s="17">
-        <v>9994008.168403117</v>
+        <v>9768604.5831468217</v>
       </c>
       <c r="D24" s="18">
-        <f t="shared" si="0"/>
-        <v>-602854.26012835838</v>
-      </c>
-      <c r="F24" s="28">
+        <f>B24-C24</f>
+        <v>-588536.73077155836</v>
+      </c>
+      <c r="F24" s="26">
         <v>160000</v>
       </c>
-      <c r="G24" s="28">
+      <c r="G24" s="26">
         <v>200000</v>
       </c>
-      <c r="H24" s="29">
+      <c r="H24" s="27">
         <v>13950</v>
       </c>
-      <c r="I24" s="30">
+      <c r="I24" s="28">
         <v>0.18</v>
       </c>
     </row>
@@ -4491,25 +4488,25 @@
         <v>2045</v>
       </c>
       <c r="B25" s="17">
-        <v>10363050.258844756</v>
+        <v>10116912.546149222</v>
       </c>
       <c r="C25" s="17">
-        <v>11024504.011576986</v>
+        <v>10761741.25121903</v>
       </c>
       <c r="D25" s="18">
-        <f t="shared" si="0"/>
-        <v>-661453.75273223035</v>
-      </c>
-      <c r="F25" s="28">
+        <f>B25-C25</f>
+        <v>-644828.70506980829</v>
+      </c>
+      <c r="F25" s="26">
         <v>200000</v>
       </c>
-      <c r="G25" s="28">
+      <c r="G25" s="26">
         <v>240000</v>
       </c>
-      <c r="H25" s="29">
+      <c r="H25" s="27">
         <v>21150</v>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="28">
         <v>0.19</v>
       </c>
     </row>
@@ -4518,25 +4515,25 @@
         <v>2046</v>
       </c>
       <c r="B26" s="17">
-        <v>11414535.571074057</v>
+        <v>11128730.197552633</v>
       </c>
       <c r="C26" s="17">
-        <v>12139095.117391396</v>
+        <v>11834064.331196917</v>
       </c>
       <c r="D26" s="18">
-        <f t="shared" si="0"/>
-        <v>-724559.54631733894</v>
-      </c>
-      <c r="F26" s="28">
+        <f>B26-C26</f>
+        <v>-705334.13364428468</v>
+      </c>
+      <c r="F26" s="26">
         <v>240000</v>
       </c>
-      <c r="G26" s="28">
+      <c r="G26" s="26">
         <v>280000</v>
       </c>
-      <c r="H26" s="29">
+      <c r="H26" s="27">
         <v>28750</v>
       </c>
-      <c r="I26" s="30">
+      <c r="I26" s="28">
         <v>0.2</v>
       </c>
     </row>
@@ -4545,25 +4542,25 @@
         <v>2047</v>
       </c>
       <c r="B27" s="17">
-        <v>12551827.238760276</v>
+        <v>12221229.535110071</v>
       </c>
       <c r="C27" s="17">
-        <v>13344345.414189417</v>
+        <v>12991597.92865763</v>
       </c>
       <c r="D27" s="18">
-        <f t="shared" si="0"/>
-        <v>-792518.17542914115</v>
-      </c>
-      <c r="F27" s="28">
+        <f>B27-C27</f>
+        <v>-770368.39354755916</v>
+      </c>
+      <c r="F27" s="26">
         <v>280000</v>
       </c>
-      <c r="G27" s="28">
+      <c r="G27" s="26">
         <v>320000</v>
       </c>
-      <c r="H27" s="29">
+      <c r="H27" s="27">
         <v>36550</v>
       </c>
-      <c r="I27" s="30">
+      <c r="I27" s="28">
         <v>0.2</v>
       </c>
     </row>
@@ -4572,25 +4569,25 @@
         <v>2048</v>
       </c>
       <c r="B28" s="17">
-        <v>13781622.713336976</v>
+        <v>13400548.525729097</v>
       </c>
       <c r="C28" s="17">
-        <v>14647291.787458716</v>
+        <v>14240785.244535789</v>
       </c>
       <c r="D28" s="18">
-        <f t="shared" si="0"/>
-        <v>-865669.07412173972</v>
-      </c>
-      <c r="F28" s="28">
+        <f>B28-C28</f>
+        <v>-840236.71880669147</v>
+      </c>
+      <c r="F28" s="26">
         <v>320000</v>
       </c>
-      <c r="G28" s="28">
+      <c r="G28" s="26">
         <v>500000</v>
       </c>
-      <c r="H28" s="29">
+      <c r="H28" s="27">
         <v>44550</v>
       </c>
-      <c r="I28" s="30">
+      <c r="I28" s="28">
         <v>0.22</v>
       </c>
     </row>
@@ -4599,25 +4596,25 @@
         <v>2049</v>
       </c>
       <c r="B29" s="17">
-        <v>15111136.459106945</v>
+        <v>14673286.541994277</v>
       </c>
       <c r="C29" s="17">
-        <v>16055453.061050788</v>
+        <v>15588492.555225791</v>
       </c>
       <c r="D29" s="18">
-        <f t="shared" si="0"/>
-        <v>-944316.60194384307</v>
-      </c>
-      <c r="F29" s="28">
+        <f>B29-C29</f>
+        <v>-915206.01323151402</v>
+      </c>
+      <c r="F29" s="26">
         <v>500000</v>
       </c>
-      <c r="G29" s="28">
+      <c r="G29" s="26">
         <v>1000000</v>
       </c>
-      <c r="H29" s="29">
+      <c r="H29" s="27">
         <v>84150</v>
       </c>
-      <c r="I29" s="30">
+      <c r="I29" s="28">
         <v>0.23</v>
       </c>
     </row>
@@ -4626,25 +4623,25 @@
         <v>2050</v>
       </c>
       <c r="B30" s="17">
-        <v>16548139.751108911</v>
+        <v>16046538.937959194</v>
       </c>
       <c r="C30" s="17">
-        <v>17577020.627284825</v>
+        <v>17042194.448823672</v>
       </c>
       <c r="D30" s="18">
-        <f t="shared" si="0"/>
-        <v>-1028880.876175914</v>
-      </c>
-      <c r="F30" s="28">
+        <f>B30-C30</f>
+        <v>-995655.5108644776</v>
+      </c>
+      <c r="F30" s="26">
         <v>1000000</v>
       </c>
-      <c r="G30" s="31">
+      <c r="G30" s="29">
         <v>100000000000</v>
       </c>
-      <c r="H30" s="29">
+      <c r="H30" s="27">
         <v>199150</v>
       </c>
-      <c r="I30" s="30">
+      <c r="I30" s="28">
         <v>0.24</v>
       </c>
     </row>
@@ -4653,14 +4650,14 @@
         <v>2051</v>
       </c>
       <c r="B31" s="17">
-        <v>18100881.988325201</v>
+        <v>17527812.667821456</v>
       </c>
       <c r="C31" s="17">
-        <v>19220817.803879041</v>
+        <v>18609926.99367414</v>
       </c>
       <c r="D31" s="18">
-        <f t="shared" si="0"/>
-        <v>-1119935.8155538402</v>
+        <f>B31-C31</f>
+        <v>-1082114.3258526847</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -4668,14 +4665,14 @@
         <v>2052</v>
       </c>
       <c r="B32" s="17">
-        <v>19778355.589390539</v>
+        <v>19125285.222171023</v>
       </c>
       <c r="C32" s="17">
-        <v>20996348.469160471</v>
+        <v>20300329.805313781</v>
       </c>
       <c r="D32" s="18">
-        <f t="shared" si="0"/>
-        <v>-1217992.8797699325</v>
+        <f>B32-C32</f>
+        <v>-1175044.5831427574</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -4683,14 +4680,14 @@
         <v>2053</v>
       </c>
       <c r="B33" s="17">
-        <v>21590258.905901067</v>
+        <v>20847760.592736922</v>
       </c>
       <c r="C33" s="17">
-        <v>22913849.438125309</v>
+        <v>22122691.262927916</v>
       </c>
       <c r="D33" s="18">
-        <f t="shared" si="0"/>
-        <v>-1323590.5322242416</v>
+        <f>B33-C33</f>
+        <v>-1274930.6701909937</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -4698,14 +4695,14 @@
         <v>2054</v>
       </c>
       <c r="B34" s="17">
-        <v>23547038.222884983</v>
+        <v>22704703.880223405</v>
       </c>
       <c r="C34" s="17">
-        <v>24984346.867037266</v>
+        <v>24086997.111078195</v>
       </c>
       <c r="D34" s="18">
-        <f t="shared" si="0"/>
-        <v>-1437308.6441522837</v>
+        <f>B34-C34</f>
+        <v>-1382293.2308547907</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -4713,14 +4710,14 @@
         <v>2055</v>
       </c>
       <c r="B35" s="17">
-        <v>25659945.317487363</v>
+        <v>24706290.820920654</v>
       </c>
       <c r="C35" s="17">
-        <v>27219716.996374957</v>
+        <v>26203982.700104926</v>
       </c>
       <c r="D35" s="18">
-        <f t="shared" si="0"/>
-        <v>-1559771.6788875945</v>
+        <f>B35-C35</f>
+        <v>-1497691.8791842721</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -4728,14 +4725,14 @@
         <v>2056</v>
       </c>
       <c r="B36" s="17">
-        <v>27941099.444769915</v>
+        <v>26863461.021234341</v>
       </c>
       <c r="C36" s="17">
-        <v>29632751.565763965</v>
+        <v>28485189.137575556</v>
       </c>
       <c r="D36" s="18">
-        <f t="shared" si="0"/>
-        <v>-1691652.1209940501</v>
+        <f>B36-C36</f>
+        <v>-1621728.1163412146</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -4743,14 +4740,14 @@
         <v>2057</v>
       </c>
       <c r="B37" s="17">
-        <v>30323269.7238805</v>
+        <v>29091108.46845638</v>
       </c>
       <c r="C37" s="17">
-        <v>31911510.161171213</v>
+        <v>30617305.54452309</v>
       </c>
       <c r="D37" s="18">
-        <f t="shared" si="0"/>
-        <v>-1588240.4372907132</v>
+        <f>B37-C37</f>
+        <v>-1526197.0760667101</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -4758,14 +4755,14 @@
         <v>2058</v>
       </c>
       <c r="B38" s="17">
-        <v>32888628.89745469</v>
+        <v>31485495.327102989</v>
       </c>
       <c r="C38" s="17">
-        <v>34365505.292565279</v>
+        <v>32909010.864530645</v>
       </c>
       <c r="D38" s="18">
-        <f t="shared" si="0"/>
-        <v>-1476876.3951105885</v>
+        <f>B38-C38</f>
+        <v>-1423515.5374276564</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -4773,14 +4770,14 @@
         <v>2059</v>
       </c>
       <c r="B39" s="17">
-        <v>35651264.191476732</v>
+        <v>34059102.042119302</v>
       </c>
       <c r="C39" s="17">
-        <v>37008212.649563551</v>
+        <v>35372250.327740766</v>
       </c>
       <c r="D39" s="18">
-        <f t="shared" si="0"/>
-        <v>-1356948.4580868185</v>
+        <f>B39-C39</f>
+        <v>-1313148.2856214643</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -4788,14 +4785,14 @@
         <v>2060</v>
       </c>
       <c r="B40" s="17">
-        <v>38626346.139609069</v>
+        <v>36825343.219754584</v>
       </c>
       <c r="C40" s="17">
-        <v>39854144.202314988</v>
+        <v>38019863.264772162</v>
       </c>
       <c r="D40" s="18">
-        <f t="shared" si="0"/>
-        <v>-1227798.0627059191</v>
+        <f>B40-C40</f>
+        <v>-1194520.0450175777</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -4803,14 +4800,14 @@
         <v>2061</v>
       </c>
       <c r="B41" s="17">
-        <v>41830211.889552779</v>
+        <v>39798637.549535871</v>
       </c>
       <c r="C41" s="17">
-        <v>42918927.89147301</v>
+        <v>40865650.030140363</v>
       </c>
       <c r="D41" s="18">
-        <f t="shared" si="0"/>
-        <v>-1088716.0019202307</v>
+        <f>B41-C41</f>
+        <v>-1067012.4806044921</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -4818,14 +4815,14 @@
         <v>2062</v>
       </c>
       <c r="B42" s="17">
-        <v>45280454.915667161</v>
+        <v>42994482.959901288</v>
       </c>
       <c r="C42" s="17">
-        <v>46219393.446327284</v>
+        <v>43924443.934896372</v>
       </c>
       <c r="D42" s="18">
-        <f t="shared" si="0"/>
-        <v>-938938.53066012263</v>
+        <f>B42-C42</f>
+        <v>-929960.97499508411</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -4833,14 +4830,14 @@
         <v>2063</v>
       </c>
       <c r="B43" s="17">
-        <v>48996021.630489737</v>
+        <v>46429537.399232559</v>
       </c>
       <c r="C43" s="17">
-        <v>49773664.802349851</v>
+        <v>47212188.563423373</v>
       </c>
       <c r="D43" s="18">
-        <f t="shared" si="0"/>
-        <v>-777643.17186011374</v>
+        <f>B43-C43</f>
+        <v>-782651.1641908139</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -4848,14 +4845,14 @@
         <v>2064</v>
       </c>
       <c r="B44" s="17">
-        <v>52997315.425682172</v>
+        <v>50121705.663347773</v>
       </c>
       <c r="C44" s="17">
-        <v>53601259.625650555</v>
+        <v>50746020.877395615</v>
       </c>
       <c r="D44" s="18">
-        <f t="shared" si="0"/>
-        <v>-603944.19996838272</v>
+        <f>B44-C44</f>
+        <v>-624315.21404784173</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -4863,14 +4860,14 @@
         <v>2065</v>
       </c>
       <c r="B45" s="17">
-        <v>57306308.713724904</v>
+        <v>54090232.722032011</v>
       </c>
       <c r="C45" s="17">
-        <v>57723196.490863077</v>
+        <v>54544360.540068679</v>
       </c>
       <c r="D45" s="18">
-        <f t="shared" si="0"/>
-        <v>-416887.77713817358</v>
+        <f>B45-C45</f>
+        <v>-454127.818036668</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -4878,14 +4875,14 @@
         <v>2066</v>
       </c>
       <c r="B46" s="17">
-        <v>61946663.585618123</v>
+        <v>58355804.031058766</v>
       </c>
       <c r="C46" s="17">
-        <v>62162110.301010445</v>
+        <v>58627005.926492825</v>
       </c>
       <c r="D46" s="18">
-        <f t="shared" si="0"/>
-        <v>-215446.71539232135</v>
+        <f>B46-C46</f>
+        <v>-271201.8954340592</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4893,14 +4890,14 @@
         <v>2067</v>
       </c>
       <c r="B47" s="19">
-        <v>66943861.747159928</v>
+        <v>62940653.352566175</v>
       </c>
       <c r="C47" s="19">
-        <v>66942376.583158143</v>
+        <v>63015237.320090815</v>
       </c>
       <c r="D47" s="20">
-        <f t="shared" si="0"/>
-        <v>1485.1640017852187</v>
+        <f>B47-C47</f>
+        <v>-74583.967524640262</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -5072,7 +5069,7 @@
         <v>15300</v>
       </c>
       <c r="F6" s="1">
-        <f t="shared" ref="F6:F48" si="0">IF((D6-E6)&lt;=20000, 0,
+        <f t="shared" ref="F6:F37" si="0">IF((D6-E6)&lt;=20000, 0,
    IF((D6-E6)&lt;=30000, ((D6-E6)-20000)*0.02,
    IF((D6-E6)&lt;=40000, 200+((D6-E6)-30000)*0.035,
    IF((D6-E6)&lt;=80000, 550+((D6-E6)-40000)*0.07,
@@ -5089,11 +5086,11 @@
       </c>
       <c r="G6" s="1">
         <f>G5*Result!$G$12+E6</f>
-        <v>31710.66372</v>
+        <v>31663.044000000002</v>
       </c>
       <c r="H6" s="1">
         <f>H5*Result!$G$13+D6-E6+F6</f>
-        <v>348676.77760000003</v>
+        <v>348335.85440000001</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -5118,11 +5115,11 @@
       </c>
       <c r="G7" s="1">
         <f>G6*Result!$G$12+E7</f>
-        <v>49312.616905027731</v>
+        <v>49162.992297119999</v>
       </c>
       <c r="H7" s="1">
         <f>H6*Result!$G$13+D7-E7+F7</f>
-        <v>548419.62179743999</v>
+        <v>547338.39310183993</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -5147,11 +5144,11 @@
       </c>
       <c r="G8" s="1">
         <f>G7*Result!$G$12+E8</f>
-        <v>68192.338116444269</v>
+        <v>67878.837001923894</v>
       </c>
       <c r="H8" s="1">
         <f>H7*Result!$G$13+D8-E8+F8</f>
-        <v>766935.20271366311</v>
+        <v>764648.78382551263</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
@@ -5176,11 +5173,11 @@
       </c>
       <c r="G9" s="1">
         <f>G8*Result!$G$12+E9</f>
-        <v>88442.583601928432</v>
+        <v>87895.058596817558</v>
       </c>
       <c r="H9" s="1">
         <f>H8*Result!$G$13+D9-E9+F9</f>
-        <v>1005723.5297223438</v>
+        <v>1001693.7552148523</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
@@ -5205,11 +5202,11 @@
       </c>
       <c r="G10" s="1">
         <f>G9*Result!$G$12+E10</f>
-        <v>110162.84300779307</v>
+        <v>109302.00726812443</v>
       </c>
       <c r="H10" s="1">
         <f>H9*Result!$G$13+D10-E10+F10</f>
-        <v>1266381.7592763919</v>
+        <v>1259988.622911084</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
@@ -5234,11 +5231,11 @@
       </c>
       <c r="G11" s="1">
         <f>G10*Result!$G$12+E11</f>
-        <v>133459.82817255199</v>
+        <v>132196.31073311373</v>
       </c>
       <c r="H11" s="1">
         <f>H10*Result!$G$13+D11-E11+F11</f>
-        <v>1550661.8284855143</v>
+        <v>1541194.0832567466</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
@@ -5263,11 +5260,11 @@
       </c>
       <c r="G12" s="1">
         <f>G11*Result!$G$12+E12</f>
-        <v>158447.99740318515</v>
+        <v>156681.31040285047</v>
       </c>
       <c r="H12" s="1">
         <f>H11*Result!$G$13+D12-E12+F12</f>
-        <v>1860451.8012552338</v>
+        <v>1847096.5385476977</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
@@ -5292,11 +5289,11 @@
       </c>
       <c r="G13" s="1">
         <f>G12*Result!$G$12+E13</f>
-        <v>185250.11780987613</v>
+        <v>182867.52784964052</v>
       </c>
       <c r="H13" s="1">
         <f>H12*Result!$G$13+D13-E13+F13</f>
-        <v>2197786.3644941282</v>
+        <v>2179617.5341803599</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
@@ -5321,11 +5318,11 @@
       </c>
       <c r="G14" s="1">
         <f>G13*Result!$G$12+E14</f>
-        <v>213997.86846197778</v>
+        <v>210873.16368463353</v>
       </c>
       <c r="H14" s="1">
         <f>H13*Result!$G$13+D14-E14+F14</f>
-        <v>2564858.1320405407</v>
+        <v>2540823.9027305744</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
@@ -5350,11 +5347,11 @@
       </c>
       <c r="G15" s="1">
         <f>G14*Result!$G$12+E15</f>
-        <v>244832.48732851705</v>
+        <v>240824.63109744186</v>
       </c>
       <c r="H15" s="1">
         <f>H14*Result!$G$13+D15-E15+F15</f>
-        <v>2964029.8184336089</v>
+        <v>2932938.6678891089</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
@@ -5379,11 +5376,11 @@
       </c>
       <c r="G16" s="1">
         <f>G15*Result!$G$12+E16</f>
-        <v>277905.46518166369</v>
+        <v>272857.12646609213</v>
       </c>
       <c r="H16" s="1">
         <f>H15*Result!$G$13+D16-E16+F16</f>
-        <v>3397847.3494310873</v>
+        <v>3358352.7651405428</v>
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
@@ -5408,11 +5405,11 @@
       </c>
       <c r="G17" s="1">
         <f>G16*Result!$G$12+E17</f>
-        <v>313379.28987231711</v>
+        <v>307115.23961295618</v>
       </c>
       <c r="H17" s="1">
         <f>H16*Result!$G$13+D17-E17+F17</f>
-        <v>3869053.9813214699</v>
+        <v>3819637.640330445</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -5437,11 +5434,11 @@
       </c>
       <c r="G18" s="1">
         <f>G17*Result!$G$12+E18</f>
-        <v>351428.2446344443</v>
+        <v>343753.60646126437</v>
       </c>
       <c r="H18" s="1">
         <f>H17*Result!$G$13+D18-E18+F18</f>
-        <v>4380588.3999881521</v>
+        <v>4319541.6852122406</v>
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
@@ -5466,11 +5463,11 @@
       </c>
       <c r="G19" s="1">
         <f>G18*Result!$G$12+E19</f>
-        <v>392239.26434024575</v>
+        <v>382937.60703819303</v>
       </c>
       <c r="H19" s="1">
         <f>H18*Result!$G$13+D19-E19+F19</f>
-        <v>4935625.2288003629</v>
+        <v>4861028.9612034997</v>
       </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
@@ -5495,11 +5492,11 @@
       </c>
       <c r="G20" s="1">
         <f>G19*Result!$G$12+E20</f>
-        <v>436012.85391293862</v>
+        <v>424844.1119752067</v>
       </c>
       <c r="H20" s="1">
         <f>H19*Result!$G$13+D20-E20+F20</f>
-        <v>5537593.1113652959</v>
+        <v>5447295.2814197671</v>
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.25">
@@ -5524,11 +5521,11 @@
       </c>
       <c r="G21" s="1">
         <f>G20*Result!$G$12+E21</f>
-        <v>482964.07340932824</v>
+        <v>469662.28087524406</v>
       </c>
       <c r="H21" s="1">
         <f>H20*Result!$G$13+D21-E21+F21</f>
-        <v>6190186.0201488752</v>
+        <v>6081777.3317536255</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
@@ -5553,11 +5550,11 @@
       </c>
       <c r="G22" s="1">
         <f>G21*Result!$G$12+E22</f>
-        <v>533323.59461188759</v>
+        <v>517594.416150456</v>
       </c>
       <c r="H22" s="1">
         <f>H21*Result!$G$13+D22-E22+F22</f>
-        <v>6897383.6935883043</v>
+        <v>6768170.7335253656</v>
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.25">
@@ -5582,11 +5579,11 @@
       </c>
       <c r="G23" s="1">
         <f>G22*Result!$G$12+E23</f>
-        <v>587338.83432139154</v>
+        <v>568856.8761845897</v>
       </c>
       <c r="H23" s="1">
         <f>H22*Result!$G$13+D23-E23+F23</f>
-        <v>7663473.6454850258</v>
+        <v>7510449.4587895209</v>
       </c>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.25">
@@ -5611,11 +5608,11 @@
       </c>
       <c r="G24" s="1">
         <f>G23*Result!$G$12+E24</f>
-        <v>645275.1699179837</v>
+        <v>623681.05194189493</v>
       </c>
       <c r="H24" s="1">
         <f>H23*Result!$G$13+D24-E24+F24</f>
-        <v>8493074.8675997984</v>
+        <v>8312886.6995568927</v>
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
@@ -5640,11 +5637,11 @@
       </c>
       <c r="G25" s="1">
         <f>G24*Result!$G$12+E25</f>
-        <v>707417.24316273793</v>
+        <v>682314.4114308178</v>
       </c>
       <c r="H25" s="1">
         <f>H24*Result!$G$13+D25-E25+F25</f>
-        <v>9391153.9082747586</v>
+        <v>9180067.8523752633</v>
       </c>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.25">
@@ -5669,11 +5666,11 @@
       </c>
       <c r="G26" s="1">
         <f>G25*Result!$G$12+E26</f>
-        <v>774070.35864530469</v>
+        <v>745021.61673703103</v>
       </c>
       <c r="H26" s="1">
         <f>H25*Result!$G$13+D26-E26+F26</f>
-        <v>10363050.258844756</v>
+        <v>10116912.546149222</v>
       </c>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.25">
@@ -5698,11 +5695,11 @@
       </c>
       <c r="G27" s="1">
         <f>G26*Result!$G$12+E27</f>
-        <v>845561.98374822806</v>
+        <v>812085.71866791998</v>
       </c>
       <c r="H27" s="1">
         <f>H26*Result!$G$13+D27-E27+F27</f>
-        <v>11414535.571074057</v>
+        <v>11128730.197552633</v>
       </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
@@ -5727,11 +5724,11 @@
       </c>
       <c r="G28" s="1">
         <f>G27*Result!$G$12+E28</f>
-        <v>922243.3574972729</v>
+        <v>883809.43440096709</v>
       </c>
       <c r="H28" s="1">
         <f>H27*Result!$G$13+D28-E28+F28</f>
-        <v>12551827.238760276</v>
+        <v>12221229.535110071</v>
       </c>
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
@@ -5759,11 +5756,11 @@
       </c>
       <c r="G29" s="1">
         <f>G28*Result!$G$12+E29</f>
-        <v>1004491.2162020579</v>
+        <v>960516.51390314626</v>
       </c>
       <c r="H29" s="1">
         <f>H28*Result!$G$13+D29-E29+F29</f>
-        <v>13781622.713336976</v>
+        <v>13400548.525729097</v>
       </c>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
@@ -5791,11 +5788,11 @@
       </c>
       <c r="G30" s="1">
         <f>G29*Result!$G$12+E30</f>
-        <v>1092709.6443650841</v>
+        <v>1042553.2012891369</v>
       </c>
       <c r="H30" s="1">
         <f>H29*Result!$G$13+D30-E30+F30</f>
-        <v>15111136.459106945</v>
+        <v>14673286.541994277</v>
       </c>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
@@ -5823,11 +5820,11 @@
       </c>
       <c r="G31" s="1">
         <f>G30*Result!$G$12+E31</f>
-        <v>1187332.0599526921</v>
+        <v>1130289.797714706</v>
       </c>
       <c r="H31" s="1">
         <f>H30*Result!$G$13+D31-E31+F31</f>
-        <v>16548139.751108911</v>
+        <v>16046538.937959194</v>
       </c>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
@@ -5855,11 +5852,11 @@
       </c>
       <c r="G32" s="1">
         <f>G31*Result!$G$12+E32</f>
-        <v>1288823.3437816019</v>
+        <v>1224122.3328599238</v>
       </c>
       <c r="H32" s="1">
         <f>H31*Result!$G$13+D32-E32+F32</f>
-        <v>18100881.988325201</v>
+        <v>17527812.667821456</v>
       </c>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
@@ -5887,11 +5884,11 @@
       </c>
       <c r="G33" s="1">
         <f>G32*Result!$G$12+E33</f>
-        <v>1397682.1234827335</v>
+        <v>1324474.3525470314</v>
       </c>
       <c r="H33" s="1">
         <f>H32*Result!$G$13+D33-E33+F33</f>
-        <v>19778355.589390539</v>
+        <v>19125285.222171023</v>
       </c>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
@@ -5919,11 +5916,11 @@
       </c>
       <c r="G34" s="1">
         <f>G33*Result!$G$12+E34</f>
-        <v>1514443.2232634416</v>
+        <v>1431798.830561999</v>
       </c>
       <c r="H34" s="1">
         <f>H33*Result!$G$13+D34-E34+F34</f>
-        <v>21590258.905901067</v>
+        <v>20847760.592736922</v>
       </c>
       <c r="K34" s="5"/>
       <c r="L34" s="5"/>
@@ -5951,11 +5948,11 @@
       </c>
       <c r="G35" s="1">
         <f>G34*Result!$G$12+E35</f>
-        <v>1639680.2915038706</v>
+        <v>1546580.2133094466</v>
       </c>
       <c r="H35" s="1">
         <f>H34*Result!$G$13+D35-E35+F35</f>
-        <v>23547038.222884983</v>
+        <v>22704703.880223405</v>
       </c>
       <c r="K35" s="5"/>
       <c r="L35" s="5"/>
@@ -5983,11 +5980,11 @@
       </c>
       <c r="G36" s="1">
         <f>G35*Result!$G$12+E36</f>
-        <v>1774008.6190968363</v>
+        <v>1669336.606530187</v>
       </c>
       <c r="H36" s="1">
         <f>H35*Result!$G$13+D36-E36+F36</f>
-        <v>25659945.317487363</v>
+        <v>24706290.820920654</v>
       </c>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
@@ -6012,11 +6009,11 @@
       </c>
       <c r="G37" s="1">
         <f>G36*Result!$G$12+E37</f>
-        <v>1918088.1623777614</v>
+        <v>1800622.1139519042</v>
       </c>
       <c r="H37" s="1">
         <f>H36*Result!$G$13+D37-E37+F37</f>
-        <v>27941099.444769915</v>
+        <v>26863461.021234341</v>
       </c>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
@@ -6032,7 +6029,7 @@
       </c>
       <c r="E38" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F38" s="1">
         <f>IF((D38-E38)*0.5&lt;=20000, 0,
@@ -6048,15 +6045,15 @@
    IF((D38-E38)*0.5&lt;=500000, 44550+((D38-E38)*0.5-320000)*0.22,
    IF((D38-E38)*0.5&lt;=1000000, 84150+((D38-E38)*0.5-500000)*0.23,
    199150+((D38-E38)*0.5-1000000)*0.24)))))))))))) * -1</f>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G38" s="1">
         <f>(G37+E38)*Result!$G$12</f>
-        <v>1798223.5594216916</v>
+        <v>1686225.5166523652</v>
       </c>
       <c r="H38" s="1">
         <f>H37*Result!$G$13+D38-E38+F38</f>
-        <v>30323269.7238805</v>
+        <v>29091108.46845638</v>
       </c>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.25">
@@ -6072,7 +6069,7 @@
       </c>
       <c r="E39" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F39" s="1">
         <f t="shared" ref="F39:F48" si="1">IF((D39-E39)*0.5&lt;=20000, 0,
@@ -6088,15 +6085,15 @@
    IF((D39-E39)*0.5&lt;=500000, 44550+((D39-E39)*0.5-320000)*0.22,
    IF((D39-E39)*0.5&lt;=1000000, 84150+((D39-E39)*0.5-500000)*0.23,
    199150+((D39-E39)*0.5-1000000)*0.24)))))))))))) * -1</f>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G39" s="1">
         <f>(G38+E39)*Result!$G$12</f>
-        <v>1669657.6972619933</v>
+        <v>1563880.6437724542</v>
       </c>
       <c r="H39" s="1">
         <f>H38*Result!$G$13+D39-E39+F39</f>
-        <v>32888628.89745469</v>
+        <v>31485495.327102989</v>
       </c>
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.25">
@@ -6112,19 +6109,19 @@
       </c>
       <c r="E40" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F40" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G40" s="1">
         <f>(G39+E40)*Result!$G$12</f>
-        <v>1531758.9306100535</v>
+        <v>1433035.2491248469</v>
       </c>
       <c r="H40" s="1">
         <f>H39*Result!$G$13+D40-E40+F40</f>
-        <v>35651264.191476732</v>
+        <v>34059102.042119302</v>
       </c>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.25">
@@ -6140,19 +6137,19 @@
       </c>
       <c r="E41" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F41" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G41" s="1">
         <f>(G40+E41)*Result!$G$12</f>
-        <v>1383849.7615298093</v>
+        <v>1293098.7164571239</v>
       </c>
       <c r="H41" s="1">
         <f>H40*Result!$G$13+D41-E41+F41</f>
-        <v>38626346.139609069</v>
+        <v>36825343.219754584</v>
       </c>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.25">
@@ -6168,19 +6165,19 @@
       </c>
       <c r="E42" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F42" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G42" s="1">
         <f>(G41+E42)*Result!$G$12</f>
-        <v>1225203.5108840244</v>
+        <v>1143439.3934996475</v>
       </c>
       <c r="H42" s="1">
         <f>H41*Result!$G$13+D42-E42+F42</f>
-        <v>41830211.889552779</v>
+        <v>39798637.549535871</v>
       </c>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.25">
@@ -6196,19 +6193,19 @@
       </c>
       <c r="E43" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F43" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G43" s="1">
         <f>(G42+E43)*Result!$G$12</f>
-        <v>1055040.7481528604</v>
+        <v>983381.74078308558</v>
       </c>
       <c r="H43" s="1">
         <f>H42*Result!$G$13+D43-E43+F43</f>
-        <v>45280454.915667161</v>
+        <v>42994482.959901288</v>
       </c>
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.25">
@@ -6224,19 +6221,19 @@
       </c>
       <c r="E44" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F44" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G44" s="1">
         <f>(G43+E44)*Result!$G$12</f>
-        <v>872525.46208441071</v>
+        <v>812203.28235577699</v>
       </c>
       <c r="H44" s="1">
         <f>H43*Result!$G$13+D44-E44+F44</f>
-        <v>48996021.630489737</v>
+        <v>46429537.399232559</v>
       </c>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.25">
@@ -6252,19 +6249,19 @@
       </c>
       <c r="E45" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F45" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G45" s="1">
         <f>(G44+E45)*Result!$G$12</f>
-        <v>676760.95336356573</v>
+        <v>629131.344636939</v>
       </c>
       <c r="H45" s="1">
         <f>H44*Result!$G$13+D45-E45+F45</f>
-        <v>52997315.425682172</v>
+        <v>50121705.663347773</v>
       </c>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.25">
@@ -6280,19 +6277,19 @@
       </c>
       <c r="E46" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F46" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G46" s="1">
         <f>(G45+E46)*Result!$G$12</f>
-        <v>466785.42911985359</v>
+        <v>433339.56868539617</v>
       </c>
       <c r="H46" s="1">
         <f>H45*Result!$G$13+D46-E46+F46</f>
-        <v>57306308.713724904</v>
+        <v>54090232.722032011</v>
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.25">
@@ -6308,19 +6305,19 @@
       </c>
       <c r="E47" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F47" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G47" s="1">
         <f>(G46+E47)*Result!$G$12</f>
-        <v>241567.27763003221</v>
+        <v>223944.18014074015</v>
       </c>
       <c r="H47" s="1">
         <f>H46*Result!$G$13+D47-E47+F47</f>
-        <v>61946663.585618123</v>
+        <v>58355804.031058766</v>
       </c>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.25">
@@ -6336,19 +6333,19 @@
       </c>
       <c r="E48" s="1">
         <f>-1*$G$37*Result!$G$6</f>
-        <v>-241567.27763003117</v>
+        <v>-223944.18014073881</v>
       </c>
       <c r="F48" s="1">
         <f t="shared" si="1"/>
-        <v>-8067.5458222523375</v>
+        <v>-7026.7903580924813</v>
       </c>
       <c r="G48" s="1">
         <f>(G47+E48)*Result!$G$12</f>
-        <v>1.1237957049161195E-9</v>
+        <v>1.4317943714559079E-9</v>
       </c>
       <c r="H48" s="1">
         <f>H47*Result!$G$13+D48-E48+F48</f>
-        <v>66943861.747159928</v>
+        <v>62940653.352566175</v>
       </c>
     </row>
   </sheetData>
@@ -6523,14 +6520,14 @@
       </c>
       <c r="H6" s="1">
         <f t="shared" ref="H6:H48" si="5">H5*$K$13+D6-E6+F6</f>
-        <v>374693.565</v>
+        <v>374326.92249999999</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>18</v>
       </c>
       <c r="K6" s="7">
         <f>Table36[[#This Row],[Value]]</f>
-        <v>0.12594169672084929</v>
+        <v>0.12437044863857565</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
@@ -6559,7 +6556,7 @@
       </c>
       <c r="H7" s="1">
         <f t="shared" si="5"/>
-        <v>588902.30014850001</v>
+        <v>587740.09264912503</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>17</v>
@@ -6595,7 +6592,7 @@
       </c>
       <c r="H8" s="1">
         <f t="shared" si="5"/>
-        <v>822954.58302991965</v>
+        <v>820498.13458391209</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>9</v>
@@ -6631,7 +6628,7 @@
       </c>
       <c r="H9" s="1">
         <f t="shared" si="5"/>
-        <v>1078443.8003849206</v>
+        <v>1074116.429877518</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>3</v>
@@ -6667,7 +6664,7 @@
       </c>
       <c r="H10" s="1">
         <f t="shared" si="5"/>
-        <v>1357087.2187529206</v>
+        <v>1350225.1347722504</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>8</v>
@@ -6703,7 +6700,7 @@
       </c>
       <c r="H11" s="1">
         <f t="shared" si="5"/>
-        <v>1660735.5377957881</v>
+        <v>1650577.7980307213</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>5</v>
@@ -6739,14 +6736,14 @@
       </c>
       <c r="H12" s="1">
         <f t="shared" si="5"/>
-        <v>1991383.1788114677</v>
+        <v>1977060.6243725044</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>6</v>
       </c>
       <c r="K12" s="7">
         <f>Table36[[#This Row],[Value]]</f>
-        <v>1.0725924</v>
+        <v>1.06948</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
@@ -6775,14 +6772,14 @@
       </c>
       <c r="H13" s="1">
         <f t="shared" si="5"/>
-        <v>2351179.3649844369</v>
+        <v>2331702.4318291536</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>7</v>
       </c>
       <c r="K13" s="7">
         <f>Table36[[#This Row],[Value]]</f>
-        <v>1.0769</v>
+        <v>1.0748500000000001</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
@@ -6811,7 +6808,7 @@
       </c>
       <c r="H14" s="1">
         <f t="shared" si="5"/>
-        <v>2742440.0542685543</v>
+        <v>2716685.3549683802</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>13</v>
@@ -6846,7 +6843,7 @@
       </c>
       <c r="H15" s="1">
         <f t="shared" si="5"/>
-        <v>3167641.7960609621</v>
+        <v>3134337.35540692</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
@@ -6875,7 +6872,7 @@
       </c>
       <c r="H16" s="1">
         <f t="shared" si="5"/>
-        <v>3629466.7138295891</v>
+        <v>3587175.7701106672</v>
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
@@ -6904,7 +6901,7 @@
       </c>
       <c r="H17" s="1">
         <f t="shared" si="5"/>
-        <v>4130809.6330476543</v>
+        <v>4077912.8054280207</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
@@ -6933,7 +6930,7 @@
       </c>
       <c r="H18" s="1">
         <f t="shared" si="5"/>
-        <v>4674789.5613320805</v>
+        <v>4609465.2464173697</v>
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
@@ -6962,7 +6959,7 @@
       </c>
       <c r="H19" s="1">
         <f t="shared" si="5"/>
-        <v>5264766.959451641</v>
+        <v>5184969.8009648332</v>
       </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
@@ -6991,7 +6988,7 @@
       </c>
       <c r="H20" s="1">
         <f t="shared" si="5"/>
-        <v>5904362.3411036571</v>
+        <v>5807799.5930372365</v>
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.25">
@@ -7020,7 +7017,7 @@
       </c>
       <c r="H21" s="1">
         <f t="shared" si="5"/>
-        <v>6597476.3036541166</v>
+        <v>6481581.8910956625</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
@@ -7049,7 +7046,7 @@
       </c>
       <c r="H22" s="1">
         <f t="shared" si="5"/>
-        <v>7348310.8584759058</v>
+        <v>7210216.9227149617</v>
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.25">
@@ -7078,7 +7075,7 @@
       </c>
       <c r="H23" s="1">
         <f t="shared" si="5"/>
-        <v>8161365.3631049069</v>
+        <v>7997871.0589923812</v>
       </c>
       <c r="J23" t="s">
         <v>19</v>
@@ -7110,7 +7107,7 @@
       </c>
       <c r="H24" s="1">
         <f t="shared" si="5"/>
-        <v>9041514.147132121</v>
+        <v>8849051.4953624085</v>
       </c>
       <c r="J24" t="s">
         <v>20</v>
@@ -7142,7 +7139,7 @@
       </c>
       <c r="H25" s="1">
         <f t="shared" si="5"/>
-        <v>9994008.168403117</v>
+        <v>9768604.5831468217</v>
       </c>
       <c r="J25" t="s">
         <v>21</v>
@@ -7174,7 +7171,7 @@
       </c>
       <c r="H26" s="1">
         <f t="shared" si="5"/>
-        <v>11024504.011576986</v>
+        <v>10761741.25121903</v>
       </c>
       <c r="J26" t="s">
         <v>11</v>
@@ -7206,7 +7203,7 @@
       </c>
       <c r="H27" s="1">
         <f t="shared" si="5"/>
-        <v>12139095.117391396</v>
+        <v>11834064.331196917</v>
       </c>
       <c r="J27" t="s">
         <v>10</v>
@@ -7238,7 +7235,7 @@
       </c>
       <c r="H28" s="1">
         <f t="shared" si="5"/>
-        <v>13344345.414189417</v>
+        <v>12991597.92865763</v>
       </c>
       <c r="J28" t="s">
         <v>12</v>
@@ -7273,7 +7270,7 @@
       </c>
       <c r="H29" s="1">
         <f t="shared" si="5"/>
-        <v>14647291.787458716</v>
+        <v>14240785.244535789</v>
       </c>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
@@ -7305,7 +7302,7 @@
       </c>
       <c r="H30" s="1">
         <f t="shared" si="5"/>
-        <v>16055453.061050788</v>
+        <v>15588492.555225791</v>
       </c>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
@@ -7337,7 +7334,7 @@
       </c>
       <c r="H31" s="1">
         <f t="shared" si="5"/>
-        <v>17577020.627284825</v>
+        <v>17042194.448823672</v>
       </c>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
@@ -7369,7 +7366,7 @@
       </c>
       <c r="H32" s="1">
         <f t="shared" si="5"/>
-        <v>19220817.803879041</v>
+        <v>18609926.99367414</v>
       </c>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
@@ -7401,7 +7398,7 @@
       </c>
       <c r="H33" s="1">
         <f t="shared" si="5"/>
-        <v>20996348.469160471</v>
+        <v>20300329.805313781</v>
       </c>
       <c r="K33" s="5"/>
       <c r="L33" s="5"/>
@@ -7433,7 +7430,7 @@
       </c>
       <c r="H34" s="1">
         <f t="shared" si="5"/>
-        <v>22913849.438125309</v>
+        <v>22122691.262927916</v>
       </c>
       <c r="K34" s="5"/>
       <c r="L34" s="5"/>
@@ -7465,7 +7462,7 @@
       </c>
       <c r="H35" s="1">
         <f t="shared" si="5"/>
-        <v>24984346.867037266</v>
+        <v>24086997.111078195</v>
       </c>
       <c r="K35" s="5"/>
       <c r="L35" s="5"/>
@@ -7497,7 +7494,7 @@
       </c>
       <c r="H36" s="1">
         <f t="shared" si="5"/>
-        <v>27219716.996374957</v>
+        <v>26203982.700104926</v>
       </c>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
@@ -7526,7 +7523,7 @@
       </c>
       <c r="H37" s="1">
         <f t="shared" si="5"/>
-        <v>29632751.565763965</v>
+        <v>28485189.137575556</v>
       </c>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
@@ -7554,7 +7551,7 @@
       </c>
       <c r="H38" s="1">
         <f t="shared" si="5"/>
-        <v>31911510.161171213</v>
+        <v>30617305.54452309</v>
       </c>
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.25">
@@ -7582,7 +7579,7 @@
       </c>
       <c r="H39" s="1">
         <f t="shared" si="5"/>
-        <v>34365505.292565279</v>
+        <v>32909010.864530645</v>
       </c>
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.25">
@@ -7610,7 +7607,7 @@
       </c>
       <c r="H40" s="1">
         <f t="shared" si="5"/>
-        <v>37008212.649563551</v>
+        <v>35372250.327740766</v>
       </c>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.25">
@@ -7638,7 +7635,7 @@
       </c>
       <c r="H41" s="1">
         <f t="shared" si="5"/>
-        <v>39854144.202314988</v>
+        <v>38019863.264772162</v>
       </c>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.25">
@@ -7666,7 +7663,7 @@
       </c>
       <c r="H42" s="1">
         <f t="shared" si="5"/>
-        <v>42918927.89147301</v>
+        <v>40865650.030140363</v>
       </c>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.25">
@@ -7694,7 +7691,7 @@
       </c>
       <c r="H43" s="1">
         <f t="shared" si="5"/>
-        <v>46219393.446327284</v>
+        <v>43924443.934896372</v>
       </c>
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.25">
@@ -7722,7 +7719,7 @@
       </c>
       <c r="H44" s="1">
         <f t="shared" si="5"/>
-        <v>49773664.802349851</v>
+        <v>47212188.563423373</v>
       </c>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.25">
@@ -7750,7 +7747,7 @@
       </c>
       <c r="H45" s="1">
         <f t="shared" si="5"/>
-        <v>53601259.625650555</v>
+        <v>50746020.877395615</v>
       </c>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.25">
@@ -7778,7 +7775,7 @@
       </c>
       <c r="H46" s="1">
         <f t="shared" si="5"/>
-        <v>57723196.490863077</v>
+        <v>54544360.540068679</v>
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.25">
@@ -7806,7 +7803,7 @@
       </c>
       <c r="H47" s="1">
         <f t="shared" si="5"/>
-        <v>62162110.301010445</v>
+        <v>58627005.926492825</v>
       </c>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.25">
@@ -7834,7 +7831,7 @@
       </c>
       <c r="H48" s="1">
         <f t="shared" si="5"/>
-        <v>66942376.583158143</v>
+        <v>63015237.320090815</v>
       </c>
     </row>
   </sheetData>

</xml_diff>